<commit_message>
working fix for first stage
</commit_message>
<xml_diff>
--- a/Model objective analysis/Capacity increase/OOB_testing/L_shape_min_unvax_35_scenarios/data/Starting_point.xlsx
+++ b/Model objective analysis/Capacity increase/OOB_testing/L_shape_min_unvax_35_scenarios/data/Starting_point.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Model objective analysis/results/OOB_testing/L_shape_min_unvax_35_scenarios/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Model objective analysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3733299E-03B3-4F29-AE5C-ABECD46A1DCE}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBD7E713-1AF3-4E4D-91B0-05E744E35DB1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13550" yWindow="-7070" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="47">
   <si>
     <t>Measles</t>
   </si>
@@ -557,7 +557,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{942AD6D9-E2BE-4540-AD66-B6783F716305}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -572,8 +572,8 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
+      <c r="A2" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -583,8 +583,8 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
+      <c r="A3" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -594,8 +594,8 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>1</v>
+      <c r="A4" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -605,42 +605,42 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>9</v>
+      <c r="A5" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
       <c r="B8">
         <v>1</v>
       </c>
@@ -649,19 +649,19 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>3</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -672,18 +672,18 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -694,453 +694,13 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13">
         <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14">
-        <v>2</v>
-      </c>
-      <c r="C14">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15">
-        <v>2</v>
-      </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B16">
-        <v>2</v>
-      </c>
-      <c r="C16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18">
-        <v>2</v>
-      </c>
-      <c r="C18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-      <c r="C19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20">
-        <v>2</v>
-      </c>
-      <c r="C20">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>6</v>
-      </c>
-      <c r="B21">
-        <v>2</v>
-      </c>
-      <c r="C21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>4</v>
-      </c>
-      <c r="B22">
-        <v>2</v>
-      </c>
-      <c r="C22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>2</v>
-      </c>
-      <c r="B23">
-        <v>2</v>
-      </c>
-      <c r="C23">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24">
-        <v>3</v>
-      </c>
-      <c r="C24">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B25">
-        <v>3</v>
-      </c>
-      <c r="C25">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>4</v>
-      </c>
-      <c r="B26">
-        <v>3</v>
-      </c>
-      <c r="C26">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27">
-        <v>4</v>
-      </c>
-      <c r="C27">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28">
-        <v>4</v>
-      </c>
-      <c r="C28">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>10</v>
-      </c>
-      <c r="B29">
-        <v>4</v>
-      </c>
-      <c r="C29">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30">
-        <v>4</v>
-      </c>
-      <c r="C30">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>2</v>
-      </c>
-      <c r="B31">
-        <v>4</v>
-      </c>
-      <c r="C31">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>5</v>
-      </c>
-      <c r="B32">
-        <v>5</v>
-      </c>
-      <c r="C32">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B33">
-        <v>5</v>
-      </c>
-      <c r="C33">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>6</v>
-      </c>
-      <c r="B34">
-        <v>5</v>
-      </c>
-      <c r="C34">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B35">
-        <v>6</v>
-      </c>
-      <c r="C35">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36">
-        <v>6</v>
-      </c>
-      <c r="C36">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>8</v>
-      </c>
-      <c r="B37">
-        <v>6</v>
-      </c>
-      <c r="C37">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38">
-        <v>7</v>
-      </c>
-      <c r="C38">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>8</v>
-      </c>
-      <c r="B39">
-        <v>7</v>
-      </c>
-      <c r="C39">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>3</v>
-      </c>
-      <c r="B40">
-        <v>7</v>
-      </c>
-      <c r="C40">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>6</v>
-      </c>
-      <c r="B41">
-        <v>7</v>
-      </c>
-      <c r="C41">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>4</v>
-      </c>
-      <c r="B42">
-        <v>7</v>
-      </c>
-      <c r="C42">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>13</v>
-      </c>
-      <c r="B43">
-        <v>8</v>
-      </c>
-      <c r="C43">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>1</v>
-      </c>
-      <c r="B44">
-        <v>8</v>
-      </c>
-      <c r="C44">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>9</v>
-      </c>
-      <c r="B45">
-        <v>8</v>
-      </c>
-      <c r="C45">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>10</v>
-      </c>
-      <c r="B46">
-        <v>8</v>
-      </c>
-      <c r="C46">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>2</v>
-      </c>
-      <c r="B47">
-        <v>8</v>
-      </c>
-      <c r="C47">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>5</v>
-      </c>
-      <c r="B48">
-        <v>9</v>
-      </c>
-      <c r="C48">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49">
-        <v>9</v>
-      </c>
-      <c r="C49">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>13</v>
-      </c>
-      <c r="B50">
-        <v>10</v>
-      </c>
-      <c r="C50">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>9</v>
-      </c>
-      <c r="B51">
-        <v>10</v>
-      </c>
-      <c r="C51">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>8</v>
-      </c>
-      <c r="B52">
-        <v>10</v>
-      </c>
-      <c r="C52">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>2</v>
-      </c>
-      <c r="B53">
-        <v>10</v>
-      </c>
-      <c r="C53">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>